<commit_message>
#7 Peripheral added in BOM
</commit_message>
<xml_diff>
--- a/Design-Files/Design-v2.0/Deliverables/BOM/Client_BOM-v2.0.xlsx
+++ b/Design-Files/Design-v2.0/Deliverables/BOM/Client_BOM-v2.0.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="243">
   <si>
     <t>#</t>
   </si>
@@ -744,6 +744,18 @@
   </si>
   <si>
     <t>32.768kHz</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>Zetiling High Power Led Chip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B07TKL2JRM </t>
+  </si>
+  <si>
+    <t>Zetiling</t>
   </si>
 </sst>
 </file>
@@ -1862,7 +1874,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
@@ -1890,7 +1902,7 @@
       <c r="J1" s="14"/>
       <c r="K1" s="14"/>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" ht="15.75" spans="1:11">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -2147,7 +2159,7 @@
       </c>
       <c r="K9" s="9"/>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" ht="15.75" spans="1:11">
       <c r="A10" s="2"/>
       <c r="B10" s="7">
         <f>ROW(B10)-ROW($B$2)</f>
@@ -2179,7 +2191,7 @@
       </c>
       <c r="K10" s="12"/>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" ht="15.75" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="7">
         <f>ROW(B11)-ROW($B$2)</f>
@@ -2243,7 +2255,7 @@
       </c>
       <c r="K12" s="12"/>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" ht="15.75" spans="1:11">
       <c r="A13" s="2"/>
       <c r="B13" s="7">
         <f>ROW(B13)-ROW($B$2)</f>
@@ -2275,7 +2287,7 @@
       </c>
       <c r="K13" s="9"/>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" ht="15.75" spans="1:11">
       <c r="A14" s="2"/>
       <c r="B14" s="7">
         <f>ROW(B14)-ROW($B$2)</f>
@@ -2309,7 +2321,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" ht="15.75" spans="1:11">
       <c r="A15" s="2"/>
       <c r="B15" s="7">
         <f>ROW(B15)-ROW($B$2)</f>
@@ -2501,7 +2513,7 @@
       </c>
       <c r="K20" s="12"/>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" ht="15.75" spans="1:11">
       <c r="A21" s="2"/>
       <c r="B21" s="7">
         <f>ROW(B21)-ROW($B$2)</f>
@@ -2565,7 +2577,7 @@
       </c>
       <c r="K22" s="12"/>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" ht="15.75" spans="1:11">
       <c r="A23" s="2"/>
       <c r="B23" s="7">
         <f>ROW(B23)-ROW($B$2)</f>
@@ -2627,7 +2639,7 @@
       </c>
       <c r="K24" s="12"/>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" ht="15.75" spans="1:11">
       <c r="A25" s="2"/>
       <c r="B25" s="7">
         <f>ROW(B25)-ROW($B$2)</f>
@@ -3141,7 +3153,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="41" spans="1:11">
+    <row r="41" ht="15.75" spans="1:11">
       <c r="A41" s="2"/>
       <c r="B41" s="7">
         <f>ROW(B41)-ROW($B$2)</f>
@@ -3173,7 +3185,7 @@
       </c>
       <c r="K41" s="9"/>
     </row>
-    <row r="42" spans="1:11">
+    <row r="42" ht="15.75" spans="1:11">
       <c r="A42" s="2"/>
       <c r="B42" s="7">
         <f>ROW(B42)-ROW($B$2)</f>
@@ -3237,7 +3249,7 @@
       </c>
       <c r="K43" s="9"/>
     </row>
-    <row r="44" spans="1:11">
+    <row r="44" ht="15.75" spans="1:11">
       <c r="A44" s="2"/>
       <c r="B44" s="7">
         <f>ROW(B44)-ROW($B$2)</f>
@@ -3333,7 +3345,7 @@
       </c>
       <c r="K46" s="12"/>
     </row>
-    <row r="47" spans="1:11">
+    <row r="47" ht="15.75" spans="1:11">
       <c r="A47" s="2"/>
       <c r="B47" s="7">
         <f>ROW(B47)-ROW($B$2)</f>
@@ -3428,6 +3440,38 @@
         <v>1</v>
       </c>
       <c r="K49" s="9"/>
+    </row>
+    <row r="50" spans="1:11">
+      <c r="A50" s="2"/>
+      <c r="B50" s="7">
+        <f>ROW(B50)-ROW($B$2)</f>
+        <v>48</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E50" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G50" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="H50" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="I50" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J50" s="9">
+        <v>10</v>
+      </c>
+      <c r="K50" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>